<commit_message>
#46 R427, R428, R429, R430, R431, R432 Added in Client BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Master-Board-v2.0/BOM/Client-BOM-Master-Board-v2.0.xlsx
+++ b/Design Files/Master-Board-v2.0/BOM/Client-BOM-Master-Board-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="695">
   <si>
     <t>#</t>
   </si>
@@ -2092,6 +2092,18 @@
   </si>
   <si>
     <t>DreamLNK</t>
+  </si>
+  <si>
+    <t>R427, R428, R429, R430, R431, R432</t>
+  </si>
+  <si>
+    <t>RES 560 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07560RL</t>
+  </si>
+  <si>
+    <t>560R</t>
   </si>
 </sst>
 </file>
@@ -2353,14 +2365,14 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2650,7 +2662,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K168"/>
+  <dimension ref="A1:K169"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="4" style="4" bestFit="1" customWidth="1"/>
@@ -2663,6 +2675,8 @@
     <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2674,9 +2688,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2746,7 +2760,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B158" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B159" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -6721,1021 +6735,1021 @@
       </c>
       <c r="K127" s="7"/>
     </row>
-    <row r="128" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1"/>
       <c r="B128" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B128" si="1">ROW(B128) - ROW($B$2)</f>
         <v>126</v>
       </c>
       <c r="C128" s="13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D128" s="9" t="s">
-        <v>167</v>
+        <v>691</v>
       </c>
       <c r="E128" s="10" t="s">
-        <v>319</v>
-      </c>
-      <c r="F128" s="7" t="s">
-        <v>652</v>
+        <v>692</v>
+      </c>
+      <c r="F128" s="9" t="s">
+        <v>395</v>
       </c>
       <c r="G128" s="10" t="s">
-        <v>398</v>
+        <v>693</v>
       </c>
       <c r="H128" s="9" t="s">
-        <v>579</v>
+        <v>540</v>
       </c>
       <c r="I128" s="10" t="s">
-        <v>655</v>
+        <v>694</v>
       </c>
       <c r="J128" s="9">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K128" s="9"/>
     </row>
-    <row r="129" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1"/>
       <c r="B129" s="11">
-        <f>ROW(B129) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>127</v>
       </c>
-      <c r="C129" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D129" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="E129" s="8" t="s">
-        <v>320</v>
+      <c r="C129" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D129" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="E129" s="10" t="s">
+        <v>319</v>
       </c>
       <c r="F129" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="G129" s="8" t="s">
-        <v>399</v>
-      </c>
-      <c r="H129" s="7" t="s">
-        <v>569</v>
+      <c r="G129" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="H129" s="9" t="s">
+        <v>579</v>
       </c>
       <c r="I129" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J129" s="7">
-        <v>1</v>
-      </c>
-      <c r="K129" s="7"/>
-    </row>
-    <row r="130" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J129" s="9">
+        <v>9</v>
+      </c>
+      <c r="K129" s="9"/>
+    </row>
+    <row r="130" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1"/>
       <c r="B130" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B130) - ROW($B$2)</f>
         <v>128</v>
       </c>
-      <c r="C130" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D130" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="E130" s="10" t="s">
-        <v>321</v>
+      <c r="C130" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D130" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E130" s="8" t="s">
+        <v>320</v>
       </c>
       <c r="F130" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="G130" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="H130" s="9" t="s">
-        <v>580</v>
+      <c r="G130" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="H130" s="7" t="s">
+        <v>569</v>
       </c>
       <c r="I130" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J130" s="9">
-        <v>1</v>
-      </c>
-      <c r="K130" s="9"/>
-    </row>
-    <row r="131" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J130" s="7">
+        <v>1</v>
+      </c>
+      <c r="K130" s="7"/>
+    </row>
+    <row r="131" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1"/>
       <c r="B131" s="11">
-        <f>ROW(B131) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>129</v>
       </c>
-      <c r="C131" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D131" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="E131" s="8" t="s">
-        <v>322</v>
+      <c r="C131" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D131" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E131" s="10" t="s">
+        <v>321</v>
       </c>
       <c r="F131" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="G131" s="8" t="s">
-        <v>400</v>
-      </c>
-      <c r="H131" s="7" t="s">
-        <v>581</v>
+      <c r="G131" s="10" t="s">
+        <v>516</v>
+      </c>
+      <c r="H131" s="9" t="s">
+        <v>580</v>
       </c>
       <c r="I131" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J131" s="7">
-        <v>1</v>
-      </c>
-      <c r="K131" s="7"/>
-    </row>
-    <row r="132" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J131" s="9">
+        <v>1</v>
+      </c>
+      <c r="K131" s="9"/>
+    </row>
+    <row r="132" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="1"/>
       <c r="B132" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B132) - ROW($B$2)</f>
         <v>130</v>
       </c>
-      <c r="C132" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D132" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="E132" s="10" t="s">
-        <v>323</v>
+      <c r="C132" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D132" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>322</v>
       </c>
       <c r="F132" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="G132" s="10" t="s">
-        <v>517</v>
-      </c>
-      <c r="H132" s="9" t="s">
-        <v>582</v>
+      <c r="G132" s="8" t="s">
+        <v>400</v>
+      </c>
+      <c r="H132" s="7" t="s">
+        <v>581</v>
       </c>
       <c r="I132" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J132" s="9">
-        <v>2</v>
-      </c>
-      <c r="K132" s="9"/>
-    </row>
-    <row r="133" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J132" s="7">
+        <v>1</v>
+      </c>
+      <c r="K132" s="7"/>
+    </row>
+    <row r="133" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="1"/>
       <c r="B133" s="11">
-        <f>ROW(B133) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>131</v>
       </c>
-      <c r="C133" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="D133" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="E133" s="8" t="s">
-        <v>324</v>
+      <c r="C133" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D133" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="E133" s="10" t="s">
+        <v>323</v>
       </c>
       <c r="F133" s="7" t="s">
-        <v>401</v>
-      </c>
-      <c r="G133" s="8" t="s">
-        <v>518</v>
-      </c>
-      <c r="H133" s="7" t="s">
-        <v>583</v>
+        <v>652</v>
+      </c>
+      <c r="G133" s="10" t="s">
+        <v>517</v>
+      </c>
+      <c r="H133" s="9" t="s">
+        <v>582</v>
       </c>
       <c r="I133" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J133" s="7">
+      <c r="J133" s="9">
         <v>2</v>
       </c>
-      <c r="K133" s="7"/>
-    </row>
-    <row r="134" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K133" s="9"/>
+    </row>
+    <row r="134" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="1"/>
       <c r="B134" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B134) - ROW($B$2)</f>
         <v>132</v>
       </c>
-      <c r="C134" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="D134" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="E134" s="10" t="s">
-        <v>325</v>
+      <c r="C134" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D134" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>324</v>
       </c>
       <c r="F134" s="7" t="s">
-        <v>652</v>
-      </c>
-      <c r="G134" s="10" t="s">
-        <v>402</v>
-      </c>
-      <c r="H134" s="9" t="s">
-        <v>584</v>
+        <v>401</v>
+      </c>
+      <c r="G134" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="H134" s="7" t="s">
+        <v>583</v>
       </c>
       <c r="I134" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J134" s="9">
-        <v>1</v>
-      </c>
-      <c r="K134" s="9"/>
+      <c r="J134" s="7">
+        <v>2</v>
+      </c>
+      <c r="K134" s="7"/>
     </row>
     <row r="135" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1"/>
       <c r="B135" s="11">
-        <f>ROW(B135) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>133</v>
       </c>
-      <c r="C135" s="12" t="s">
+      <c r="C135" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D135" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="E135" s="8" t="s">
-        <v>326</v>
+      <c r="D135" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="E135" s="10" t="s">
+        <v>325</v>
       </c>
       <c r="F135" s="7" t="s">
-        <v>403</v>
-      </c>
-      <c r="G135" s="8" t="s">
-        <v>519</v>
-      </c>
-      <c r="H135" s="7" t="s">
-        <v>585</v>
+        <v>652</v>
+      </c>
+      <c r="G135" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="H135" s="9" t="s">
+        <v>584</v>
       </c>
       <c r="I135" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J135" s="7">
-        <v>1</v>
-      </c>
-      <c r="K135" s="7"/>
-    </row>
-    <row r="136" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J135" s="9">
+        <v>1</v>
+      </c>
+      <c r="K135" s="9"/>
+    </row>
+    <row r="136" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1"/>
       <c r="B136" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B136) - ROW($B$2)</f>
         <v>134</v>
       </c>
-      <c r="C136" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="D136" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="E136" s="10" t="s">
-        <v>327</v>
-      </c>
-      <c r="F136" s="9" t="s">
-        <v>404</v>
-      </c>
-      <c r="G136" s="10" t="s">
-        <v>520</v>
-      </c>
-      <c r="H136" s="9" t="s">
-        <v>553</v>
+      <c r="C136" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D136" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="E136" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="F136" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="G136" s="8" t="s">
+        <v>519</v>
+      </c>
+      <c r="H136" s="7" t="s">
+        <v>585</v>
       </c>
       <c r="I136" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J136" s="9">
-        <v>3</v>
-      </c>
-      <c r="K136" s="9"/>
+      <c r="J136" s="7">
+        <v>1</v>
+      </c>
+      <c r="K136" s="7"/>
     </row>
     <row r="137" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="1"/>
       <c r="B137" s="11">
-        <f>ROW(B137) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>135</v>
       </c>
-      <c r="C137" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D137" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="E137" s="8" t="s">
-        <v>328</v>
-      </c>
-      <c r="F137" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="G137" s="8" t="s">
-        <v>405</v>
-      </c>
-      <c r="H137" s="7" t="s">
-        <v>586</v>
+      <c r="C137" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D137" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E137" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="F137" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="G137" s="10" t="s">
+        <v>520</v>
+      </c>
+      <c r="H137" s="9" t="s">
+        <v>553</v>
       </c>
       <c r="I137" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J137" s="7">
-        <v>8</v>
-      </c>
-      <c r="K137" s="7"/>
-    </row>
-    <row r="138" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J137" s="9">
+        <v>3</v>
+      </c>
+      <c r="K137" s="9"/>
+    </row>
+    <row r="138" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1"/>
       <c r="B138" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B138) - ROW($B$2)</f>
         <v>136</v>
       </c>
-      <c r="C138" s="13" t="s">
+      <c r="C138" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D138" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="E138" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="F138" s="9" t="s">
-        <v>406</v>
-      </c>
-      <c r="G138" s="10" t="s">
-        <v>521</v>
-      </c>
-      <c r="H138" s="9" t="s">
-        <v>585</v>
+      <c r="D138" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="F138" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="G138" s="8" t="s">
+        <v>405</v>
+      </c>
+      <c r="H138" s="7" t="s">
+        <v>586</v>
       </c>
       <c r="I138" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J138" s="9">
-        <v>4</v>
-      </c>
-      <c r="K138" s="9"/>
+      <c r="J138" s="7">
+        <v>8</v>
+      </c>
+      <c r="K138" s="7"/>
     </row>
     <row r="139" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="1"/>
       <c r="B139" s="11">
-        <f>ROW(B139) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>137</v>
       </c>
-      <c r="C139" s="12" t="s">
+      <c r="C139" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D139" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="E139" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="F139" s="7" t="s">
-        <v>407</v>
-      </c>
-      <c r="G139" s="8" t="s">
-        <v>522</v>
-      </c>
-      <c r="H139" s="7" t="s">
+      <c r="D139" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="E139" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="F139" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G139" s="10" t="s">
+        <v>521</v>
+      </c>
+      <c r="H139" s="9" t="s">
         <v>585</v>
       </c>
       <c r="I139" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J139" s="7">
-        <v>2</v>
-      </c>
-      <c r="K139" s="7"/>
-    </row>
-    <row r="140" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J139" s="9">
+        <v>4</v>
+      </c>
+      <c r="K139" s="9"/>
+    </row>
+    <row r="140" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="1"/>
       <c r="B140" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B140) - ROW($B$2)</f>
         <v>138</v>
       </c>
-      <c r="C140" s="13" t="s">
+      <c r="C140" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D140" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="E140" s="10" t="s">
-        <v>331</v>
-      </c>
-      <c r="F140" s="9" t="s">
-        <v>404</v>
-      </c>
-      <c r="G140" s="10" t="s">
-        <v>523</v>
-      </c>
-      <c r="H140" s="9" t="s">
+      <c r="D140" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="E140" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F140" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="G140" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="H140" s="7" t="s">
         <v>585</v>
       </c>
       <c r="I140" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J140" s="9">
-        <v>1</v>
-      </c>
-      <c r="K140" s="9"/>
-    </row>
-    <row r="141" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J140" s="7">
+        <v>2</v>
+      </c>
+      <c r="K140" s="7"/>
+    </row>
+    <row r="141" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A141" s="1"/>
       <c r="B141" s="11">
-        <f>ROW(B141) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>139</v>
       </c>
-      <c r="C141" s="12" t="s">
+      <c r="C141" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D141" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="E141" s="8" t="s">
-        <v>332</v>
-      </c>
-      <c r="F141" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="G141" s="8" t="s">
-        <v>524</v>
-      </c>
-      <c r="H141" s="7" t="s">
+      <c r="D141" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="E141" s="10" t="s">
+        <v>331</v>
+      </c>
+      <c r="F141" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="G141" s="10" t="s">
+        <v>523</v>
+      </c>
+      <c r="H141" s="9" t="s">
         <v>585</v>
       </c>
       <c r="I141" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J141" s="7">
-        <v>1</v>
-      </c>
-      <c r="K141" s="7"/>
+      <c r="J141" s="9">
+        <v>1</v>
+      </c>
+      <c r="K141" s="9"/>
     </row>
     <row r="142" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A142" s="1"/>
       <c r="B142" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B142) - ROW($B$2)</f>
         <v>140</v>
       </c>
-      <c r="C142" s="13" t="s">
+      <c r="C142" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D142" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="E142" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="F142" s="9" t="s">
-        <v>409</v>
-      </c>
-      <c r="G142" s="10" t="s">
-        <v>525</v>
-      </c>
-      <c r="H142" s="9" t="s">
-        <v>551</v>
+      <c r="D142" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E142" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="F142" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="G142" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="H142" s="7" t="s">
+        <v>585</v>
       </c>
       <c r="I142" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J142" s="9">
-        <v>1</v>
-      </c>
-      <c r="K142" s="9"/>
+      <c r="J142" s="7">
+        <v>1</v>
+      </c>
+      <c r="K142" s="7"/>
     </row>
     <row r="143" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A143" s="1"/>
       <c r="B143" s="11">
-        <f>ROW(B143) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>141</v>
       </c>
-      <c r="C143" s="12" t="s">
+      <c r="C143" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D143" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="E143" s="8" t="s">
-        <v>334</v>
-      </c>
-      <c r="F143" s="7" t="s">
-        <v>410</v>
-      </c>
-      <c r="G143" s="8" t="s">
-        <v>526</v>
-      </c>
-      <c r="H143" s="7" t="s">
-        <v>587</v>
+      <c r="D143" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="E143" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="F143" s="9" t="s">
+        <v>409</v>
+      </c>
+      <c r="G143" s="10" t="s">
+        <v>525</v>
+      </c>
+      <c r="H143" s="9" t="s">
+        <v>551</v>
       </c>
       <c r="I143" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J143" s="7">
-        <v>1</v>
-      </c>
-      <c r="K143" s="7"/>
+      <c r="J143" s="9">
+        <v>1</v>
+      </c>
+      <c r="K143" s="9"/>
     </row>
     <row r="144" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="1"/>
       <c r="B144" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B144) - ROW($B$2)</f>
         <v>142</v>
       </c>
-      <c r="C144" s="13" t="s">
+      <c r="C144" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D144" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="E144" s="10" t="s">
-        <v>335</v>
-      </c>
-      <c r="F144" s="9" t="s">
-        <v>406</v>
-      </c>
-      <c r="G144" s="10" t="s">
-        <v>527</v>
-      </c>
-      <c r="H144" s="9" t="s">
+      <c r="D144" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E144" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="F144" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="G144" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="H144" s="7" t="s">
         <v>587</v>
       </c>
       <c r="I144" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J144" s="9">
-        <v>1</v>
-      </c>
-      <c r="K144" s="9"/>
+      <c r="J144" s="7">
+        <v>1</v>
+      </c>
+      <c r="K144" s="7"/>
     </row>
     <row r="145" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="1"/>
       <c r="B145" s="11">
-        <f>ROW(B145) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>143</v>
       </c>
-      <c r="C145" s="12" t="s">
+      <c r="C145" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D145" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="E145" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F145" s="7" t="s">
-        <v>411</v>
-      </c>
-      <c r="G145" s="8" t="s">
-        <v>528</v>
-      </c>
-      <c r="H145" s="7" t="s">
-        <v>551</v>
+      <c r="D145" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="E145" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="F145" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G145" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="H145" s="9" t="s">
+        <v>587</v>
       </c>
       <c r="I145" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J145" s="7">
-        <v>1</v>
-      </c>
-      <c r="K145" s="7"/>
+      <c r="J145" s="9">
+        <v>1</v>
+      </c>
+      <c r="K145" s="9"/>
     </row>
     <row r="146" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="1"/>
       <c r="B146" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B146) - ROW($B$2)</f>
         <v>144</v>
       </c>
-      <c r="C146" s="13" t="s">
+      <c r="C146" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D146" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="E146" s="10" t="s">
-        <v>337</v>
-      </c>
-      <c r="F146" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="G146" s="10" t="s">
-        <v>529</v>
-      </c>
-      <c r="H146" s="9" t="s">
+      <c r="D146" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="E146" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="F146" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="G146" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="H146" s="7" t="s">
         <v>551</v>
       </c>
       <c r="I146" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J146" s="9">
-        <v>1</v>
-      </c>
-      <c r="K146" s="9"/>
+      <c r="J146" s="7">
+        <v>1</v>
+      </c>
+      <c r="K146" s="7"/>
     </row>
     <row r="147" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="1"/>
       <c r="B147" s="11">
-        <f>ROW(B147) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>145</v>
       </c>
-      <c r="C147" s="12" t="s">
+      <c r="C147" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D147" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="E147" s="8" t="s">
-        <v>338</v>
-      </c>
-      <c r="F147" s="7" t="s">
-        <v>413</v>
-      </c>
-      <c r="G147" s="8" t="s">
-        <v>530</v>
-      </c>
-      <c r="H147" s="7" t="s">
-        <v>585</v>
+      <c r="D147" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="E147" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="F147" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="G147" s="10" t="s">
+        <v>529</v>
+      </c>
+      <c r="H147" s="9" t="s">
+        <v>551</v>
       </c>
       <c r="I147" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J147" s="7">
-        <v>2</v>
-      </c>
-      <c r="K147" s="7"/>
+      <c r="J147" s="9">
+        <v>1</v>
+      </c>
+      <c r="K147" s="9"/>
     </row>
     <row r="148" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="1"/>
       <c r="B148" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B148) - ROW($B$2)</f>
         <v>146</v>
       </c>
-      <c r="C148" s="13" t="s">
+      <c r="C148" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D148" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="E148" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="F148" s="9" t="s">
-        <v>406</v>
-      </c>
-      <c r="G148" s="10" t="s">
-        <v>531</v>
-      </c>
-      <c r="H148" s="9" t="s">
+      <c r="D148" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="E148" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="F148" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="G148" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="H148" s="7" t="s">
         <v>585</v>
       </c>
       <c r="I148" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J148" s="9">
-        <v>3</v>
-      </c>
-      <c r="K148" s="9"/>
+      <c r="J148" s="7">
+        <v>2</v>
+      </c>
+      <c r="K148" s="7"/>
     </row>
     <row r="149" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="1"/>
       <c r="B149" s="11">
-        <f>ROW(B149) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>147</v>
       </c>
-      <c r="C149" s="12" t="s">
+      <c r="C149" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D149" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="E149" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="F149" s="7" t="s">
-        <v>414</v>
-      </c>
-      <c r="G149" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="H149" s="7" t="s">
-        <v>587</v>
+      <c r="D149" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="E149" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="F149" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G149" s="10" t="s">
+        <v>531</v>
+      </c>
+      <c r="H149" s="9" t="s">
+        <v>585</v>
       </c>
       <c r="I149" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J149" s="7">
-        <v>1</v>
-      </c>
-      <c r="K149" s="7"/>
+      <c r="J149" s="9">
+        <v>3</v>
+      </c>
+      <c r="K149" s="9"/>
     </row>
     <row r="150" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1"/>
       <c r="B150" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B150) - ROW($B$2)</f>
         <v>148</v>
       </c>
-      <c r="C150" s="13"/>
-      <c r="D150" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="E150" s="10" t="s">
-        <v>340</v>
-      </c>
-      <c r="F150" s="9" t="s">
-        <v>653</v>
-      </c>
-      <c r="G150" s="10" t="s">
-        <v>415</v>
-      </c>
-      <c r="H150" s="9" t="s">
-        <v>550</v>
+      <c r="C150" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D150" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E150" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="F150" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="G150" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="H150" s="7" t="s">
+        <v>587</v>
       </c>
       <c r="I150" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J150" s="9">
-        <v>1</v>
-      </c>
-      <c r="K150" s="9"/>
+      <c r="J150" s="7">
+        <v>1</v>
+      </c>
+      <c r="K150" s="7"/>
     </row>
     <row r="151" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="1"/>
       <c r="B151" s="11">
-        <f>ROW(B151) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>149</v>
       </c>
-      <c r="C151" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D151" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="E151" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="F151" s="7" t="s">
-        <v>416</v>
-      </c>
-      <c r="G151" s="8" t="s">
-        <v>533</v>
-      </c>
-      <c r="H151" s="7" t="s">
-        <v>585</v>
+      <c r="C151" s="13"/>
+      <c r="D151" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="E151" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="F151" s="9" t="s">
+        <v>653</v>
+      </c>
+      <c r="G151" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="H151" s="9" t="s">
+        <v>550</v>
       </c>
       <c r="I151" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J151" s="7">
-        <v>1</v>
-      </c>
-      <c r="K151" s="7"/>
-    </row>
-    <row r="152" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J151" s="9">
+        <v>1</v>
+      </c>
+      <c r="K151" s="9"/>
+    </row>
+    <row r="152" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="1"/>
       <c r="B152" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B152) - ROW($B$2)</f>
         <v>150</v>
       </c>
-      <c r="C152" s="13" t="s">
+      <c r="C152" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D152" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="E152" s="10" t="s">
-        <v>342</v>
-      </c>
-      <c r="F152" s="9" t="s">
-        <v>417</v>
-      </c>
-      <c r="G152" s="10" t="s">
-        <v>534</v>
-      </c>
-      <c r="H152" s="9" t="s">
-        <v>588</v>
+      <c r="D152" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="E152" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="F152" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="G152" s="8" t="s">
+        <v>533</v>
+      </c>
+      <c r="H152" s="7" t="s">
+        <v>585</v>
       </c>
       <c r="I152" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J152" s="9">
-        <v>1</v>
-      </c>
-      <c r="K152" s="9"/>
-    </row>
-    <row r="153" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J152" s="7">
+        <v>1</v>
+      </c>
+      <c r="K152" s="7"/>
+    </row>
+    <row r="153" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="1"/>
       <c r="B153" s="11">
-        <f>ROW(B153) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>151</v>
       </c>
-      <c r="C153" s="12" t="s">
+      <c r="C153" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D153" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="E153" s="8" t="s">
-        <v>343</v>
-      </c>
-      <c r="F153" s="7" t="s">
-        <v>404</v>
-      </c>
-      <c r="G153" s="8" t="s">
-        <v>535</v>
-      </c>
-      <c r="H153" s="7" t="s">
-        <v>589</v>
+      <c r="D153" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="E153" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="F153" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="G153" s="10" t="s">
+        <v>534</v>
+      </c>
+      <c r="H153" s="9" t="s">
+        <v>588</v>
       </c>
       <c r="I153" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J153" s="7">
-        <v>1</v>
-      </c>
-      <c r="K153" s="7"/>
-    </row>
-    <row r="154" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J153" s="9">
+        <v>1</v>
+      </c>
+      <c r="K153" s="9"/>
+    </row>
+    <row r="154" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1"/>
       <c r="B154" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B154) - ROW($B$2)</f>
         <v>152</v>
       </c>
-      <c r="C154" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D154" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="E154" s="10" t="s">
-        <v>344</v>
-      </c>
-      <c r="F154" s="9" t="s">
-        <v>418</v>
-      </c>
-      <c r="G154" s="10" t="s">
-        <v>536</v>
-      </c>
-      <c r="H154" s="9" t="s">
-        <v>590</v>
+      <c r="C154" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D154" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="E154" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="F154" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="G154" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="H154" s="7" t="s">
+        <v>589</v>
       </c>
       <c r="I154" s="10" t="s">
-        <v>647</v>
-      </c>
-      <c r="J154" s="9">
-        <v>1</v>
-      </c>
-      <c r="K154" s="9"/>
+        <v>655</v>
+      </c>
+      <c r="J154" s="7">
+        <v>1</v>
+      </c>
+      <c r="K154" s="7"/>
     </row>
     <row r="155" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A155" s="1"/>
       <c r="B155" s="11">
-        <f>ROW(B155) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>153</v>
       </c>
-      <c r="C155" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D155" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="E155" s="15" t="s">
-        <v>345</v>
-      </c>
-      <c r="F155" s="14" t="s">
-        <v>652</v>
-      </c>
-      <c r="G155" s="15" t="s">
-        <v>419</v>
-      </c>
-      <c r="H155" s="14" t="s">
-        <v>591</v>
-      </c>
-      <c r="I155" s="15" t="s">
-        <v>608</v>
-      </c>
-      <c r="J155" s="14">
-        <v>1</v>
-      </c>
-      <c r="K155" s="16" t="s">
-        <v>654</v>
-      </c>
+      <c r="C155" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D155" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="E155" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="F155" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="G155" s="10" t="s">
+        <v>536</v>
+      </c>
+      <c r="H155" s="9" t="s">
+        <v>590</v>
+      </c>
+      <c r="I155" s="10" t="s">
+        <v>647</v>
+      </c>
+      <c r="J155" s="9">
+        <v>1</v>
+      </c>
+      <c r="K155" s="9"/>
     </row>
     <row r="156" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A156" s="1"/>
       <c r="B156" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B156) - ROW($B$2)</f>
         <v>154</v>
       </c>
-      <c r="C156" s="13" t="s">
+      <c r="C156" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D156" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="E156" s="10" t="s">
+      <c r="D156" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="E156" s="15" t="s">
         <v>345</v>
       </c>
-      <c r="F156" s="7" t="s">
+      <c r="F156" s="14" t="s">
         <v>652</v>
       </c>
-      <c r="G156" s="10" t="s">
+      <c r="G156" s="15" t="s">
         <v>419</v>
       </c>
-      <c r="H156" s="9" t="s">
+      <c r="H156" s="14" t="s">
         <v>591</v>
       </c>
-      <c r="I156" s="10" t="s">
-        <v>647</v>
-      </c>
-      <c r="J156" s="9">
-        <v>1</v>
-      </c>
-      <c r="K156" s="9"/>
+      <c r="I156" s="15" t="s">
+        <v>608</v>
+      </c>
+      <c r="J156" s="14">
+        <v>1</v>
+      </c>
+      <c r="K156" s="16" t="s">
+        <v>654</v>
+      </c>
     </row>
     <row r="157" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A157" s="1"/>
       <c r="B157" s="11">
-        <f>ROW(B157) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>155</v>
       </c>
-      <c r="C157" s="12"/>
-      <c r="D157" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="E157" s="8" t="s">
-        <v>346</v>
+      <c r="C157" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D157" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="E157" s="10" t="s">
+        <v>345</v>
       </c>
       <c r="F157" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="G157" s="8" t="s">
-        <v>537</v>
-      </c>
-      <c r="H157" s="7" t="s">
-        <v>592</v>
-      </c>
-      <c r="I157" s="8" t="s">
-        <v>648</v>
-      </c>
-      <c r="J157" s="7">
-        <v>1</v>
-      </c>
-      <c r="K157" s="7"/>
-    </row>
-    <row r="158" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G157" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="H157" s="9" t="s">
+        <v>591</v>
+      </c>
+      <c r="I157" s="10" t="s">
+        <v>647</v>
+      </c>
+      <c r="J157" s="9">
+        <v>1</v>
+      </c>
+      <c r="K157" s="9"/>
+    </row>
+    <row r="158" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A158" s="1"/>
       <c r="B158" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B158) - ROW($B$2)</f>
         <v>156</v>
       </c>
-      <c r="C158" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="D158" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="E158" s="10" t="s">
-        <v>347</v>
-      </c>
-      <c r="F158" s="9" t="s">
-        <v>420</v>
-      </c>
-      <c r="G158" s="10" t="s">
-        <v>538</v>
-      </c>
-      <c r="H158" s="9" t="s">
-        <v>593</v>
-      </c>
-      <c r="I158" s="10" t="s">
-        <v>647</v>
-      </c>
-      <c r="J158" s="9">
-        <v>1</v>
-      </c>
-      <c r="K158" s="9"/>
+      <c r="C158" s="12"/>
+      <c r="D158" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="E158" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="F158" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="G158" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="H158" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="I158" s="8" t="s">
+        <v>648</v>
+      </c>
+      <c r="J158" s="7">
+        <v>1</v>
+      </c>
+      <c r="K158" s="7"/>
     </row>
     <row r="159" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B159" s="11">
-        <f t="shared" ref="B159" si="1">ROW(B159) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>157</v>
       </c>
       <c r="C159" s="13" t="s">
-        <v>661</v>
+        <v>40</v>
       </c>
       <c r="D159" s="9" t="s">
-        <v>10</v>
+        <v>197</v>
       </c>
       <c r="E159" s="10" t="s">
-        <v>662</v>
+        <v>347</v>
       </c>
       <c r="F159" s="9" t="s">
-        <v>652</v>
+        <v>420</v>
       </c>
       <c r="G159" s="10" t="s">
-        <v>663</v>
+        <v>538</v>
       </c>
       <c r="H159" s="9" t="s">
-        <v>557</v>
+        <v>593</v>
       </c>
       <c r="I159" s="10" t="s">
-        <v>655</v>
+        <v>647</v>
       </c>
       <c r="J159" s="9">
         <v>1</v>
@@ -7744,85 +7758,85 @@
     </row>
     <row r="160" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B160" s="11">
-        <f>ROW(B160) - ROW($B$2)</f>
+        <f t="shared" ref="B160" si="2">ROW(B160) - ROW($B$2)</f>
         <v>158</v>
       </c>
       <c r="C160" s="13" t="s">
         <v>661</v>
       </c>
-      <c r="D160" s="7" t="s">
-        <v>664</v>
-      </c>
-      <c r="E160" s="8" t="s">
-        <v>665</v>
+      <c r="D160" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E160" s="10" t="s">
+        <v>662</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>652</v>
       </c>
-      <c r="G160" s="8" t="s">
-        <v>666</v>
-      </c>
-      <c r="H160" s="7" t="s">
-        <v>569</v>
+      <c r="G160" s="10" t="s">
+        <v>663</v>
+      </c>
+      <c r="H160" s="9" t="s">
+        <v>557</v>
       </c>
       <c r="I160" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J160" s="7">
-        <v>7</v>
-      </c>
-      <c r="K160" s="7"/>
-    </row>
-    <row r="161" spans="2:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J160" s="9">
+        <v>1</v>
+      </c>
+      <c r="K160" s="9"/>
+    </row>
+    <row r="161" spans="2:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B161" s="11">
-        <f t="shared" ref="B161:B162" si="2">ROW(B161) - ROW($B$2)</f>
+        <f>ROW(B161) - ROW($B$2)</f>
         <v>159</v>
       </c>
       <c r="C161" s="13" t="s">
         <v>661</v>
       </c>
       <c r="D161" s="7" t="s">
-        <v>679</v>
+        <v>664</v>
       </c>
       <c r="E161" s="8" t="s">
-        <v>680</v>
+        <v>665</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>652</v>
       </c>
       <c r="G161" s="8" t="s">
-        <v>681</v>
+        <v>666</v>
       </c>
       <c r="H161" s="7" t="s">
-        <v>655</v>
+        <v>569</v>
       </c>
       <c r="I161" s="10" t="s">
         <v>655</v>
       </c>
       <c r="J161" s="7">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K161" s="7"/>
     </row>
-    <row r="162" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B162" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="B162:B163" si="3">ROW(B162) - ROW($B$2)</f>
         <v>160</v>
       </c>
       <c r="C162" s="13" t="s">
         <v>661</v>
       </c>
       <c r="D162" s="7" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="E162" s="8" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>652</v>
       </c>
       <c r="G162" s="8" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="H162" s="7" t="s">
         <v>655</v>
@@ -7837,80 +7851,78 @@
     </row>
     <row r="163" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B163" s="11">
-        <f t="shared" ref="B163:B167" si="3">ROW(B163) - ROW($B$2)</f>
+        <f t="shared" si="3"/>
         <v>161</v>
       </c>
       <c r="C163" s="13" t="s">
         <v>661</v>
       </c>
-      <c r="D163" s="9" t="s">
-        <v>667</v>
-      </c>
-      <c r="E163" s="10" t="s">
-        <v>655</v>
+      <c r="D163" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="E163" s="8" t="s">
+        <v>683</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>652</v>
       </c>
-      <c r="G163" s="10" t="s">
-        <v>668</v>
-      </c>
-      <c r="H163" s="9" t="s">
-        <v>669</v>
+      <c r="G163" s="8" t="s">
+        <v>684</v>
+      </c>
+      <c r="H163" s="7" t="s">
+        <v>655</v>
       </c>
       <c r="I163" s="10" t="s">
         <v>655</v>
       </c>
-      <c r="J163" s="9">
-        <v>1</v>
-      </c>
-      <c r="K163" s="21" t="s">
-        <v>670</v>
-      </c>
+      <c r="J163" s="7">
+        <v>1</v>
+      </c>
+      <c r="K163" s="7"/>
     </row>
     <row r="164" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B164" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="B164:B168" si="4">ROW(B164) - ROW($B$2)</f>
         <v>162</v>
       </c>
       <c r="C164" s="13" t="s">
         <v>661</v>
       </c>
-      <c r="D164" s="7" t="s">
-        <v>671</v>
-      </c>
-      <c r="E164" s="8" t="s">
+      <c r="D164" s="9" t="s">
+        <v>667</v>
+      </c>
+      <c r="E164" s="10" t="s">
         <v>655</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>652</v>
       </c>
-      <c r="G164" s="8" t="s">
-        <v>672</v>
+      <c r="G164" s="10" t="s">
+        <v>668</v>
       </c>
       <c r="H164" s="9" t="s">
         <v>669</v>
       </c>
-      <c r="I164" s="8" t="s">
-        <v>655</v>
-      </c>
-      <c r="J164" s="7">
-        <v>4</v>
-      </c>
-      <c r="K164" s="22" t="s">
+      <c r="I164" s="10" t="s">
+        <v>655</v>
+      </c>
+      <c r="J164" s="9">
+        <v>1</v>
+      </c>
+      <c r="K164" s="20" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="165" spans="2:11" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B165" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>163</v>
       </c>
       <c r="C165" s="13" t="s">
         <v>661</v>
       </c>
       <c r="D165" s="7" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="E165" s="8" t="s">
         <v>655</v>
@@ -7919,72 +7931,74 @@
         <v>652</v>
       </c>
       <c r="G165" s="8" t="s">
-        <v>655</v>
-      </c>
-      <c r="H165" s="7" t="s">
-        <v>655</v>
+        <v>672</v>
+      </c>
+      <c r="H165" s="9" t="s">
+        <v>669</v>
       </c>
       <c r="I165" s="8" t="s">
         <v>655</v>
       </c>
-      <c r="J165" s="7"/>
-      <c r="K165" s="19" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="166" spans="2:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J165" s="7">
+        <v>4</v>
+      </c>
+      <c r="K165" s="21" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="166" spans="2:11" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B166" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>164</v>
       </c>
       <c r="C166" s="13" t="s">
         <v>661</v>
       </c>
       <c r="D166" s="7" t="s">
-        <v>655</v>
+        <v>673</v>
       </c>
       <c r="E166" s="8" t="s">
-        <v>686</v>
+        <v>655</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>652</v>
       </c>
       <c r="G166" s="8" t="s">
-        <v>685</v>
+        <v>655</v>
       </c>
       <c r="H166" s="7" t="s">
-        <v>687</v>
+        <v>655</v>
       </c>
       <c r="I166" s="8" t="s">
         <v>655</v>
       </c>
-      <c r="J166" s="7">
-        <v>1</v>
-      </c>
-      <c r="K166" s="19"/>
-    </row>
-    <row r="167" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J166" s="7"/>
+      <c r="K166" s="19" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="167" spans="2:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B167" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>165</v>
       </c>
       <c r="C167" s="13" t="s">
         <v>661</v>
       </c>
       <c r="D167" s="7" t="s">
-        <v>688</v>
+        <v>655</v>
       </c>
       <c r="E167" s="8" t="s">
-        <v>655</v>
+        <v>686</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>652</v>
       </c>
       <c r="G167" s="8" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="H167" s="7" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="I167" s="8" t="s">
         <v>655</v>
@@ -7994,36 +8008,67 @@
       </c>
       <c r="K167" s="19"/>
     </row>
-    <row r="168" spans="2:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B168" s="11">
-        <f>ROW(B168) - ROW($B$2)</f>
+        <f t="shared" si="4"/>
         <v>166</v>
       </c>
       <c r="C168" s="13" t="s">
         <v>661</v>
       </c>
       <c r="D168" s="7" t="s">
-        <v>675</v>
+        <v>688</v>
       </c>
       <c r="E168" s="8" t="s">
-        <v>676</v>
+        <v>655</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>652</v>
       </c>
       <c r="G168" s="8" t="s">
+        <v>689</v>
+      </c>
+      <c r="H168" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="I168" s="8" t="s">
+        <v>655</v>
+      </c>
+      <c r="J168" s="7">
+        <v>1</v>
+      </c>
+      <c r="K168" s="19"/>
+    </row>
+    <row r="169" spans="2:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B169" s="11">
+        <f>ROW(B169) - ROW($B$2)</f>
+        <v>167</v>
+      </c>
+      <c r="C169" s="13" t="s">
+        <v>661</v>
+      </c>
+      <c r="D169" s="7" t="s">
+        <v>675</v>
+      </c>
+      <c r="E169" s="8" t="s">
+        <v>676</v>
+      </c>
+      <c r="F169" s="9" t="s">
+        <v>652</v>
+      </c>
+      <c r="G169" s="8" t="s">
         <v>677</v>
       </c>
-      <c r="H168" s="7" t="s">
-        <v>655</v>
-      </c>
-      <c r="I168" s="8" t="s">
-        <v>655</v>
-      </c>
-      <c r="J168" s="7">
-        <v>1</v>
-      </c>
-      <c r="K168" s="19" t="s">
+      <c r="H169" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="I169" s="8" t="s">
+        <v>655</v>
+      </c>
+      <c r="J169" s="7">
+        <v>1</v>
+      </c>
+      <c r="K169" s="19" t="s">
         <v>678</v>
       </c>
     </row>
@@ -8032,8 +8077,8 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K163" r:id="rId1"/>
-    <hyperlink ref="K164" r:id="rId2"/>
+    <hyperlink ref="K164" r:id="rId1"/>
+    <hyperlink ref="K165" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>